<commit_message>
Cutelaria: descritivo refeito com o arquivo correto
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sSyyX8JcyBNahLXt6A2aR
</commit_message>
<xml_diff>
--- a/CUTELARIA_descritivo.xlsx
+++ b/CUTELARIA_descritivo.xlsx
@@ -1674,10 +1674,10 @@
         <v>12</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>CORTADOR DE UNHA UNHEX BLISTER 12UN</t>
+          <t>CORTADOR DE UNHA UNHEX BLISTER 12X1UN</t>
         </is>
       </c>
     </row>
@@ -1869,10 +1869,10 @@
         <v>12</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>ALICATES DE CUTICULA BONI PINCA PONTA RETA 12UN</t>
+          <t>ALICATES DE CUTICULA BONI PINCA PONTA RETA 12X1UN</t>
         </is>
       </c>
     </row>
@@ -18171,10 +18171,10 @@
         <v>1</v>
       </c>
       <c r="F434" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G434" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H434" s="2" t="inlineStr">
         <is>
@@ -18183,7 +18183,7 @@
       </c>
       <c r="I434" t="inlineStr">
         <is>
-          <t>DISCO KATY UNHA</t>
+          <t>DISCO KATY UNHA 1UN</t>
         </is>
       </c>
     </row>
@@ -48084,10 +48084,10 @@
         <v>1</v>
       </c>
       <c r="F1201" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G1201" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H1201" s="2" t="inlineStr">
         <is>
@@ -48096,7 +48096,7 @@
       </c>
       <c r="I1201" t="inlineStr">
         <is>
-          <t>BISTURI DE CALOS MERHEJE DORSAL</t>
+          <t>BISTURI DE CALOS MERHEJE DORSAL 1UN</t>
         </is>
       </c>
     </row>
@@ -55845,10 +55845,10 @@
         <v>1</v>
       </c>
       <c r="F1400" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G1400" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H1400" s="2" t="inlineStr">
         <is>
@@ -55857,7 +55857,7 @@
       </c>
       <c r="I1400" t="inlineStr">
         <is>
-          <t>ALICATES DE CUTICULA PANVEL ACESS</t>
+          <t>ALICATES DE CUTICULA PANVEL ACESS 1UN</t>
         </is>
       </c>
     </row>
@@ -71150,11 +71150,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1792">
-    <sortState ref="A2:H1792">
-      <sortCondition descending="1" ref="A1"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:H1792"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>